<commit_message>
Primeira vez passando para algém testar
</commit_message>
<xml_diff>
--- a/modelos/modelo.xlsx
+++ b/modelos/modelo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luari\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0025527C-B6CE-4A4C-8666-788A72AD4071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{0025527C-B6CE-4A4C-8666-788A72AD4071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45A66082-E256-40C3-AD58-0DD2C60349FF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{231199EE-4300-4F8B-A0B3-A2B2F5200136}"/>
   </bookViews>
@@ -266,13 +266,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -285,6 +279,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -680,226 +680,221 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="29.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7"/>
-      <c r="B1" s="9" t="s">
+      <c r="A1" s="5"/>
+      <c r="B1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
     </row>
     <row r="2" spans="1:6" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
+      <c r="A2" s="6"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
     </row>
     <row r="3" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
     </row>
     <row r="4" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
     </row>
     <row r="5" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
     </row>
     <row r="6" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
     </row>
     <row r="8" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
     </row>
     <row r="9" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
     </row>
     <row r="11" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
     </row>
     <row r="12" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
     </row>
     <row r="13" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
     </row>
     <row r="14" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
     </row>
     <row r="15" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
     </row>
     <row r="16" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
     </row>
     <row r="17" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
     </row>
     <row r="18" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
     </row>
     <row r="19" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
     </row>
     <row r="20" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
     </row>
     <row r="21" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="5"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
+      <c r="A21" s="4"/>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
     </row>
     <row r="22" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="5"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
+      <c r="A22" s="4"/>
+      <c r="B22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B18:F18"/>
     <mergeCell ref="B20:F22"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="B19:F19"/>
@@ -916,6 +911,11 @@
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B18:F18"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.47" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" scale="62" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
Comecei a colocar a câmera começando pelo ícone dela
</commit_message>
<xml_diff>
--- a/modelos/modelo.xlsx
+++ b/modelos/modelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/484c53c37b433491/Desktop/Projetos/Transformers - Convertedor de arquivos/modelos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="8_{0025527C-B6CE-4A4C-8666-788A72AD4071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C752E14-FCFB-49E1-BCD0-DD8FDF297A14}"/>
+  <xr:revisionPtr revIDLastSave="119" documentId="8_{0025527C-B6CE-4A4C-8666-788A72AD4071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E6AAA04-B87A-4D45-88E1-FCD1594C4C50}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{231199EE-4300-4F8B-A0B3-A2B2F5200136}"/>
   </bookViews>
@@ -50,34 +50,7 @@
     <t>CLIENTE</t>
   </si>
   <si>
-    <t>PADRÃO</t>
-  </si>
-  <si>
-    <t>FILME/OP</t>
-  </si>
-  <si>
-    <t>OP TUBETE</t>
-  </si>
-  <si>
-    <t>PESO PALETE</t>
-  </si>
-  <si>
-    <t>PESO TOTAL</t>
-  </si>
-  <si>
-    <t>PESO LÍQUIDO</t>
-  </si>
-  <si>
     <t>OPERADOR</t>
-  </si>
-  <si>
-    <t>SOBRA</t>
-  </si>
-  <si>
-    <t>MÁQUINA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PESO TUBETE </t>
   </si>
   <si>
     <r>
@@ -147,19 +120,46 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">Nº DO PALETE           </t>
+  </si>
+  <si>
+    <t>MÁQUINA</t>
+  </si>
+  <si>
+    <t>PESO LÍQUIDO</t>
+  </si>
+  <si>
     <t>PERDA OPERACIONAL</t>
   </si>
   <si>
     <t>PERDA MECÂNICA</t>
   </si>
   <si>
-    <t>TOTAL BOBINA  /CAIXA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nº DO PALETE           </t>
+    <t>SOBRA</t>
+  </si>
+  <si>
+    <t>PESO TOTAL</t>
   </si>
   <si>
     <t>OBS</t>
+  </si>
+  <si>
+    <t>PADRÃO</t>
+  </si>
+  <si>
+    <t>FILME/OP</t>
+  </si>
+  <si>
+    <t>OP TUBETE</t>
+  </si>
+  <si>
+    <t>PESO PALETE</t>
+  </si>
+  <si>
+    <t>TOTAL BOBINA /CAIXA</t>
+  </si>
+  <si>
+    <t>PESO TUBETE</t>
   </si>
 </sst>
 </file>
@@ -218,7 +218,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -251,19 +251,47 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -277,29 +305,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -368,6 +405,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -690,261 +731,257 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr defaultRowHeight="31.5" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="33" style="1" customWidth="1"/>
+    <col min="1" max="1" width="34.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="76.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="29.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9"/>
-      <c r="B1" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
+      <c r="A1" s="8"/>
+      <c r="B1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
     </row>
     <row r="2" spans="1:11" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
+      <c r="A2" s="9"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
     </row>
     <row r="3" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
     </row>
     <row r="4" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
+      <c r="A5" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
     </row>
     <row r="7" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
+        <v>13</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
     </row>
     <row r="8" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
+        <v>14</v>
+      </c>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
     </row>
     <row r="9" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
+      <c r="A9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
     </row>
     <row r="10" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+    </row>
+    <row r="12" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+    </row>
+    <row r="13" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="12"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="14"/>
+    </row>
+    <row r="14" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="K14" s="4"/>
+    </row>
+    <row r="15" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="12"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="14"/>
+      <c r="K15" s="4"/>
+    </row>
+    <row r="16" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="12"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="14"/>
+      <c r="K16" s="4"/>
+    </row>
+    <row r="17" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="12"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="14"/>
+      <c r="K17" s="4"/>
+    </row>
+    <row r="18" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="12"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="14"/>
+      <c r="K18" s="4"/>
+    </row>
+    <row r="19" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+    </row>
+    <row r="20" spans="1:11" ht="187.5" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A20" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-    </row>
-    <row r="11" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-    </row>
-    <row r="12" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-    </row>
-    <row r="13" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-    </row>
-    <row r="14" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="K14" s="4"/>
-    </row>
-    <row r="15" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-    </row>
-    <row r="16" spans="1:11" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-    </row>
-    <row r="17" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-    </row>
-    <row r="18" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-    </row>
-    <row r="19" spans="1:6" s="3" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-    </row>
-    <row r="20" spans="1:6" ht="187.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A20" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-    </row>
-    <row r="21" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A21" s="6"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+    </row>
+    <row r="21" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A21" s="5"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
     </row>
-    <row r="22" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A22" s="7"/>
+    <row r="22" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A22" s="5"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
     </row>
-    <row r="23" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A23" s="7"/>
+    <row r="23" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A23" s="5"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
     </row>
-    <row r="24" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A24" s="7"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-    </row>
-    <row r="25" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="7"/>
+    <row r="24" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="20">
     <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B18:F18"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B18:F18"/>
     <mergeCell ref="B19:F19"/>
     <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F16"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="A1:A2"/>
@@ -955,7 +992,7 @@
     <mergeCell ref="B1:F2"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.47" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" scale="57" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="58" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>